<commit_message>
Refined script that adds flags before staging
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friday" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_16_W" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_21_M" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_22_Tu" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_10_Th" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -525,6 +527,188 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>KBH</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>29</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1000,7 +1184,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Improved logic for a c flag
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28695" yWindow="-16320" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Trades" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_16_W" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_21_M" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_22_Tu" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_10_Th" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_12_M" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_1_Th" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_6_Tu" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_23_W" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_25_F" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_29_Tu" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_30_W" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -624,6 +630,204 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>FDX</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>STZ</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -657,7 +861,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>DRI</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -666,7 +870,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -682,7 +886,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>SNX</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -691,7 +895,230 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>CCL</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>JBL</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ACN</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -1184,7 +1611,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
More flagging logic and paste values
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" tabRatio="600" firstSheet="3" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Trades" sheetId="1" state="visible" r:id="rId1"/>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
REvised stage trades to not hard code trade size when staging in AM
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" tabRatio="600" firstSheet="3" activeTab="7" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="3" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Trades" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,16 +13,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wednesday" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thursday" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friday" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_16_W" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_21_M" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_22_Tu" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_12_M" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_1_Th" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_6_Tu" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_23_W" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_25_F" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_29_Tu" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_30_W" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_21_M" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_22_Tu" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_12_M" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_1_Th" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_6_Tu" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_23_W" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_25_F" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_29_Tu" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_30_W" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -539,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -572,7 +571,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>KBH</t>
+          <t>FDX</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -581,7 +580,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -589,31 +588,6 @@
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>PAYX</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>MOC</t>
         </is>
@@ -663,16 +637,16 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>FDX</t>
+          <t>NKE</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>long</t>
+          <t>short</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -729,7 +703,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>NKE</t>
+          <t>STZ</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -738,7 +712,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -757,6 +731,97 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>IBKR Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>DRI</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>SNX</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -795,7 +860,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>STZ</t>
+          <t>CCL</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -804,7 +869,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>12</v>
+        <v>63</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -812,97 +877,6 @@
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>DRI</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>SNX</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>MOC</t>
         </is>
@@ -952,16 +926,16 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>CCL</t>
+          <t>JBL</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -980,72 +954,6 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>IBKR Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>JBL</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1093,7 +1001,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -1118,7 +1026,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -1536,16 +1444,16 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>LEN</t>
+          <t>MLKN</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -1569,7 +1477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1602,7 +1510,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>MLKN</t>
+          <t>KBH</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -1611,7 +1519,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -1619,6 +1527,31 @@
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>PAYX</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>MOC</t>
         </is>

</xml_diff>

<commit_message>
Flagging improvements and quieted diffs
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/58c6644054d92bd9/repos/Trading_Algo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_B16AC8868EE5093B7FE34CB66CF3F875ED0C05E2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_89F114CFC47829604C96C4465582196A5E6394CB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E3575B4-59FF-4DF8-AE76-E9AB8BA7F4D2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11760" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="816" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily_Trades" sheetId="1" r:id="rId1"/>
@@ -20,22 +20,38 @@
     <sheet name="Wednesday" sheetId="5" r:id="rId5"/>
     <sheet name="Thursday" sheetId="6" r:id="rId6"/>
     <sheet name="Friday" sheetId="7" r:id="rId7"/>
-    <sheet name="9_21_M" sheetId="8" r:id="rId8"/>
-    <sheet name="9_22_Tu" sheetId="9" r:id="rId9"/>
-    <sheet name="10_12_M" sheetId="10" r:id="rId10"/>
-    <sheet name="10_1_Th" sheetId="11" r:id="rId11"/>
-    <sheet name="10_6_Tu" sheetId="12" r:id="rId12"/>
-    <sheet name="9_23_W" sheetId="13" r:id="rId13"/>
-    <sheet name="9_25_F" sheetId="14" r:id="rId14"/>
-    <sheet name="9_29_Tu" sheetId="15" r:id="rId15"/>
-    <sheet name="9_30_W" sheetId="16" r:id="rId16"/>
+    <sheet name="10_6_Tu" sheetId="8" r:id="rId8"/>
+    <sheet name="10_7_W" sheetId="13" r:id="rId9"/>
+    <sheet name="10_8_Th" sheetId="14" r:id="rId10"/>
+    <sheet name="10_12_M" sheetId="9" r:id="rId11"/>
+    <sheet name="10_13_Tu" sheetId="10" r:id="rId12"/>
+    <sheet name="10_14_W" sheetId="11" r:id="rId13"/>
+    <sheet name="10_15_Th" sheetId="12" r:id="rId14"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="38">
+  <si>
+    <t>Trade Mode</t>
+  </si>
+  <si>
+    <t>Full_Auto</t>
+  </si>
+  <si>
+    <t>Trade Modes:</t>
+  </si>
+  <si>
+    <t>"Single Day", or</t>
+  </si>
+  <si>
+    <t>"Multiday", or</t>
+  </si>
+  <si>
+    <t>"Full_Auto"</t>
+  </si>
   <si>
     <t>Ticker</t>
   </si>
@@ -52,7 +68,7 @@
     <t>ToS Exit</t>
   </si>
   <si>
-    <t>MLKN</t>
+    <t>ADBE</t>
   </si>
   <si>
     <t>long</t>
@@ -64,67 +80,73 @@
     <t>MOC</t>
   </si>
   <si>
-    <t>Trade Mode</t>
-  </si>
-  <si>
-    <t>Full_Auto</t>
-  </si>
-  <si>
-    <t>Trade Modes:</t>
-  </si>
-  <si>
-    <t>"Single Day", or</t>
-  </si>
-  <si>
-    <t>"Multiday", or</t>
-  </si>
-  <si>
-    <t>"Full_Auto"</t>
-  </si>
-  <si>
-    <t>ADBE</t>
-  </si>
-  <si>
     <t>ORCL</t>
   </si>
   <si>
     <t>KR</t>
   </si>
   <si>
-    <t>KBH</t>
-  </si>
-  <si>
-    <t>PAYX</t>
-  </si>
-  <si>
-    <t>FDX</t>
-  </si>
-  <si>
-    <t>NKE</t>
+    <t>STZ</t>
   </si>
   <si>
     <t>short</t>
   </si>
   <si>
-    <t>STZ</t>
-  </si>
-  <si>
-    <t>DRI</t>
-  </si>
-  <si>
-    <t>SNX</t>
-  </si>
-  <si>
-    <t>CCL</t>
-  </si>
-  <si>
-    <t>JBL</t>
-  </si>
-  <si>
-    <t>MU</t>
-  </si>
-  <si>
-    <t>ACN</t>
+    <t>C</t>
+  </si>
+  <si>
+    <t>GS</t>
+  </si>
+  <si>
+    <t>JNJ</t>
+  </si>
+  <si>
+    <t>JPM</t>
+  </si>
+  <si>
+    <t>WFC</t>
+  </si>
+  <si>
+    <t>ASML</t>
+  </si>
+  <si>
+    <t>BAC</t>
+  </si>
+  <si>
+    <t>BLK</t>
+  </si>
+  <si>
+    <t>FAST</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>STT</t>
+  </si>
+  <si>
+    <t>BNY</t>
+  </si>
+  <si>
+    <t>PNC</t>
+  </si>
+  <si>
+    <t>SCHW</t>
+  </si>
+  <si>
+    <t>SNA</t>
+  </si>
+  <si>
+    <t>USB</t>
+  </si>
+  <si>
+    <t>AA</t>
+  </si>
+  <si>
+    <t>PEP</t>
+  </si>
+  <si>
+    <t>DAL</t>
   </si>
 </sst>
 </file>
@@ -539,19 +561,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -560,42 +582,42 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -604,42 +626,110 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:E2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1">
-        <v>39</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -648,252 +738,283 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1">
+        <v>24</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>27</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1">
+        <v>8</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="1">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1">
+        <v>14</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1">
+        <v>23</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="1">
-        <v>63</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <v>8</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -914,32 +1035,32 @@
   <sheetData>
     <row r="2" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C2" s="3" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C8" s="5" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C9" s="4" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C10" s="4" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C11" s="4" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -961,19 +1082,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -994,19 +1115,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1027,19 +1148,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1060,70 +1181,70 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1">
         <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C3" s="1">
         <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1">
         <v>25</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1144,19 +1265,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1171,36 +1292,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1209,59 +1330,42 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:E3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="C2" s="1">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="1">
-        <v>12</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Imrpoved staging to save files once and not hidden
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28695" yWindow="-16320" windowWidth="29040" windowHeight="16440" tabRatio="816" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="816" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Trades" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,10 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wednesday" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thursday" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friday" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_14_W" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_15_Th" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_16_F" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_19_M" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_15_Th" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_16_F" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_19_M" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_20_Tu" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_21_W" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -538,11 +539,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -579,30 +577,330 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>STLD</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>ALLY</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>EFX</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
           <t>short</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
-        <v>27</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="C4" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>short</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>KEY</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>NOC</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
         </is>
       </c>
     </row>
@@ -655,7 +953,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>COF</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -664,7 +962,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -685,7 +983,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>ALLY</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -694,7 +992,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -715,16 +1013,16 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
@@ -738,14 +1036,14 @@
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>GE</t>
+          <t>OMC</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -754,7 +1052,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
@@ -775,7 +1073,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>PEGA</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -784,7 +1082,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
@@ -805,7 +1103,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>UAL</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -814,7 +1112,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
@@ -835,7 +1133,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -844,7 +1142,7 @@
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
@@ -865,7 +1163,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>KEY</t>
+          <t>CME</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -874,7 +1172,7 @@
         </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
@@ -895,7 +1193,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>MMM</t>
+          <t>DHR</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -904,7 +1202,7 @@
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
@@ -925,7 +1223,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>NOC</t>
+          <t>PM</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -934,7 +1232,7 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
@@ -955,16 +1253,16 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>PNR</t>
+          <t>TMO</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
@@ -978,14 +1276,14 @@
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>WAB</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -994,19 +1292,515 @@
         </is>
       </c>
       <c r="C13" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction (ToS_Open)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ToS_Open_Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Direction (ToS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>CSX</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>LUV</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>LVS</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>PKG</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>AAL</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>115</v>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>BX</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>CMCSA</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>DOV</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>HBAN</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>long</t>
         </is>
@@ -1409,180 +2203,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="20.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="10" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="14.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="7.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="14.28515625" bestFit="1" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Direction (ToS_Open)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Share Size</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ToS_Open_Exit</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>ToS Exit</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Direction (ToS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>BNY</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>PNC</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>SCHW</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>USB</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1634,11 +2254,11 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -1652,7 +2272,7 @@
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
@@ -1664,7 +2284,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
@@ -1682,7 +2302,7 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
@@ -1694,7 +2314,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
@@ -1712,7 +2332,7 @@
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
@@ -1724,7 +2344,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
@@ -1742,7 +2362,7 @@
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
@@ -1754,7 +2374,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
@@ -1772,7 +2392,7 @@
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
@@ -1784,7 +2404,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C7" s="1" t="n">
@@ -1802,7 +2422,86 @@
       </c>
       <c r="F7" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction (ToS_Open)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Share Size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ToS_Open_Exit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>ToS Exit</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Direction (ToS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>FITB</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>27</v>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Changed my cancel all script to be able to choose which account(s)
</commit_message>
<xml_diff>
--- a/Live_Trade_Info.xlsx
+++ b/Live_Trade_Info.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="816" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="816" firstSheet="0" activeTab="8" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily_Trades" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,11 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wednesday" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thursday" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friday" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_15_Th" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_16_F" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_19_M" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_20_Tu" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_21_W" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_20_Tu" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_21_W" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_22_Th" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_26_M" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_27_Tu" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>ALLY</t>
+          <t>DECK</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -637,16 +637,16 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>EFX</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
@@ -660,14 +660,14 @@
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>long</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>GE</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -697,7 +697,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>AXP</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
@@ -749,156 +749,6 @@
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>KEY</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>68</v>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>MMM</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>NOC</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>RTX</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>long</t>
         </is>
@@ -915,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -953,7 +803,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>COF</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -962,7 +812,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -983,7 +833,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>CTOS</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -992,7 +842,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>3</v>
+        <v>145</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -1013,7 +863,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>NFLX</t>
+          <t>NUE</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -1022,7 +872,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
@@ -1043,7 +893,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>OMC</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -1052,7 +902,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
@@ -1073,7 +923,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>PEGA</t>
+          <t>ECL</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -1082,7 +932,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
@@ -1103,7 +953,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>UAL</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -1112,7 +962,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
@@ -1133,7 +983,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
@@ -1142,7 +992,7 @@
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
@@ -1163,7 +1013,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>HCA</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -1172,7 +1022,7 @@
         </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
@@ -1193,7 +1043,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>DHR</t>
+          <t>HLT</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -1202,7 +1052,7 @@
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
@@ -1223,7 +1073,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>PM</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
@@ -1232,7 +1082,7 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
@@ -1253,7 +1103,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>TMO</t>
+          <t>IQV</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -1262,7 +1112,7 @@
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
@@ -1283,7 +1133,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>WAB</t>
+          <t>ITW</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -1305,6 +1155,336 @@
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>JCI</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>PCAR</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>PNR</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>22</v>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>RCL</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>SHW</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="n">
+        <v>87</v>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>SPGI</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>UPS</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>XYL</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>long</t>
         </is>
@@ -1321,7 +1501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1359,7 +1539,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>BKR</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -1368,7 +1548,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -1389,7 +1569,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>ENPH</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -1398,7 +1578,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -1411,396 +1591,6 @@
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>LRCX</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>LUV</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>LVS</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E7" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F7" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>PKG</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>TXN</t>
-        </is>
-      </c>
-      <c r="B10" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E10" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>AAL</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="n">
-        <v>115</v>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>BX</t>
-        </is>
-      </c>
-      <c r="B12" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E12" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>CMCSA</t>
-        </is>
-      </c>
-      <c r="B13" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="n">
-        <v>62</v>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F13" s="1" t="inlineStr">
-        <is>
-          <t>short</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>DOV</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>DOW</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C15" s="1" t="n">
-        <v>46</v>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E15" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F15" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>HBAN</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>long</t>
-        </is>
-      </c>
-      <c r="C16" s="1" t="n">
-        <v>90</v>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E16" s="1" t="inlineStr">
-        <is>
-          <t>MOC</t>
-        </is>
-      </c>
-      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>long</t>
         </is>
@@ -2203,16 +1993,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="20.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="10" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="14.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="7.85546875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="14.28515625" bestFit="1" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -2249,7 +2031,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>COF</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -2258,7 +2040,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -2279,7 +2061,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
@@ -2288,7 +2070,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -2309,7 +2091,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>JBHT</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
@@ -2318,7 +2100,7 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
@@ -2339,7 +2121,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>CFG</t>
+          <t>OMC</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -2348,7 +2130,7 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
@@ -2369,7 +2151,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>MTB</t>
+          <t>PEGA</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
@@ -2378,7 +2160,7 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
@@ -2399,7 +2181,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>TFC</t>
+          <t>UAL</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
@@ -2408,7 +2190,7 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
@@ -2421,6 +2203,186 @@
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>ABT</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>CME</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>DHR</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>TMO</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>WAB</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>long</t>
         </is>
@@ -2437,11 +2399,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -2478,7 +2437,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>CSX</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -2487,7 +2446,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
@@ -2500,6 +2459,726 @@
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>LUV</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>LVS</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>PKG</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>TXN</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>AAL</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>113</v>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>BX</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>CMCSA</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>DOV</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>HBAN</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>LMT</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>NSC</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>PHM</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>SNA</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>TSCO</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>UNP</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="1" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>long</t>
         </is>

</xml_diff>